<commit_message>
Add Tribal Digital Masqs and Extend Your Session feature
</commit_message>
<xml_diff>
--- a/source/spreadsheets/BES_NV_Environments_and_Features_for_Claude.xlsx
+++ b/source/spreadsheets/BES_NV_Environments_and_Features_for_Claude.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmestes87/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD6ECE5C-99C1-5746-9BE3-A69AA353DC2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB597A0-2936-1F44-8353-862480EF2412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31320" yWindow="600" windowWidth="24620" windowHeight="20300" xr2:uid="{DB342F5B-931C-1D4F-B9D1-BF0B938CA362}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17960" xr2:uid="{DB342F5B-931C-1D4F-B9D1-BF0B938CA362}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
   <si>
     <t>Requires Subscription</t>
   </si>
@@ -222,6 +222,9 @@
   </si>
   <si>
     <t>Requires SuperTouch</t>
+  </si>
+  <si>
+    <t>Extend Your Session</t>
   </si>
 </sst>
 </file>
@@ -602,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D87255-3CFF-534A-B67C-04E80AB8E4B8}">
-  <dimension ref="A2:G57"/>
+  <dimension ref="A2:G58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
@@ -1688,111 +1691,111 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B52">
         <v>1</v>
       </c>
       <c r="C52">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
       <c r="E52">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F52">
         <v>0</v>
       </c>
       <c r="G52">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B53">
         <v>1</v>
       </c>
       <c r="C53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D53">
         <v>1</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F53">
         <v>0</v>
       </c>
       <c r="G53">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B54">
         <v>1</v>
       </c>
       <c r="C54">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D54">
         <v>1</v>
       </c>
       <c r="E54">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F54">
         <v>0</v>
       </c>
       <c r="G54">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B55">
         <v>1</v>
       </c>
       <c r="C55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D55">
         <v>1</v>
       </c>
       <c r="E55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F55">
         <v>0</v>
       </c>
       <c r="G55">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B56">
         <v>1</v>
       </c>
       <c r="C56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D56">
         <v>1</v>
       </c>
       <c r="E56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F56">
         <v>0</v>
@@ -1803,24 +1806,47 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
+        <v>36</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="C57">
+        <v>0</v>
+      </c>
+      <c r="D57">
+        <v>1</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>0</v>
+      </c>
+      <c r="G57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
         <v>55</v>
       </c>
-      <c r="B57">
-        <v>1</v>
-      </c>
-      <c r="C57">
-        <v>0</v>
-      </c>
-      <c r="D57">
-        <v>1</v>
-      </c>
-      <c r="E57">
-        <v>0</v>
-      </c>
-      <c r="F57">
-        <v>0</v>
-      </c>
-      <c r="G57">
+      <c r="B58">
+        <v>1</v>
+      </c>
+      <c r="C58">
+        <v>0</v>
+      </c>
+      <c r="D58">
+        <v>1</v>
+      </c>
+      <c r="E58">
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <v>0</v>
+      </c>
+      <c r="G58">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add vane-style Environment/Feature counters, extend SuperTouch to Neoverse
</commit_message>
<xml_diff>
--- a/source/spreadsheets/BES_NV_Environments_and_Features_for_Claude.xlsx
+++ b/source/spreadsheets/BES_NV_Environments_and_Features_for_Claude.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmestes87/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB597A0-2936-1F44-8353-862480EF2412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4213A8AF-0D29-8749-AD2A-1F37610292E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17960" xr2:uid="{DB342F5B-931C-1D4F-B9D1-BF0B938CA362}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" xr2:uid="{DB342F5B-931C-1D4F-B9D1-BF0B938CA362}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
   <si>
     <t>Requires Subscription</t>
   </si>
@@ -225,6 +225,12 @@
   </si>
   <si>
     <t>Extend Your Session</t>
+  </si>
+  <si>
+    <t>Environment</t>
+  </si>
+  <si>
+    <t>Feature</t>
   </si>
 </sst>
 </file>
@@ -605,13 +611,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D87255-3CFF-534A-B67C-04E80AB8E4B8}">
-  <dimension ref="A2:G58"/>
+  <dimension ref="A2:I58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -633,8 +639,14 @@
       <c r="G2" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -656,8 +668,14 @@
       <c r="G3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>41</v>
       </c>
@@ -679,8 +697,14 @@
       <c r="G4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -702,8 +726,14 @@
       <c r="G5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -725,8 +755,14 @@
       <c r="G6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -748,8 +784,14 @@
       <c r="G7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -771,8 +813,14 @@
       <c r="G8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -794,8 +842,14 @@
       <c r="G9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -817,8 +871,14 @@
       <c r="G10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>44</v>
       </c>
@@ -840,8 +900,14 @@
       <c r="G11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -863,8 +929,14 @@
       <c r="G12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H12">
+        <v>1</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -886,8 +958,14 @@
       <c r="G13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H13">
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -909,8 +987,14 @@
       <c r="G14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -932,8 +1016,14 @@
       <c r="G15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -955,8 +1045,14 @@
       <c r="G16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -978,8 +1074,14 @@
       <c r="G17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -1001,8 +1103,14 @@
       <c r="G18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H18">
+        <v>1</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>40</v>
       </c>
@@ -1024,8 +1132,14 @@
       <c r="G19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H19">
+        <v>1</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -1047,8 +1161,14 @@
       <c r="G20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H20">
+        <v>1</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -1070,8 +1190,14 @@
       <c r="G21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H21">
+        <v>1</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>39</v>
       </c>
@@ -1093,8 +1219,14 @@
       <c r="G22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H22">
+        <v>1</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>7</v>
       </c>
@@ -1116,8 +1248,14 @@
       <c r="G23">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H23">
+        <v>1</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>20</v>
       </c>
@@ -1139,8 +1277,14 @@
       <c r="G24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H24">
+        <v>1</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -1162,8 +1306,14 @@
       <c r="G25">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H25">
+        <v>1</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -1185,8 +1335,14 @@
       <c r="G26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>11</v>
       </c>
@@ -1208,13 +1364,19 @@
       <c r="G27">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H27">
+        <v>1</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>1</v>
       </c>
@@ -1236,8 +1398,14 @@
       <c r="G29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H29">
+        <v>1</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>50</v>
       </c>
@@ -1259,8 +1427,14 @@
       <c r="G30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H30">
+        <v>1</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>52</v>
       </c>
@@ -1282,8 +1456,14 @@
       <c r="G31">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H31">
+        <v>1</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>51</v>
       </c>
@@ -1305,8 +1485,14 @@
       <c r="G32">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H32">
+        <v>1</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>49</v>
       </c>
@@ -1328,13 +1514,19 @@
       <c r="G33">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H33">
+        <v>1</v>
+      </c>
+      <c r="I33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>25</v>
       </c>
@@ -1356,8 +1548,14 @@
       <c r="G35">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H35">
+        <v>1</v>
+      </c>
+      <c r="I35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>31</v>
       </c>
@@ -1379,8 +1577,14 @@
       <c r="G36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H36">
+        <v>1</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>32</v>
       </c>
@@ -1402,8 +1606,14 @@
       <c r="G37">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H37">
+        <v>1</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>27</v>
       </c>
@@ -1425,8 +1635,14 @@
       <c r="G38">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H38">
+        <v>1</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>26</v>
       </c>
@@ -1448,13 +1664,19 @@
       <c r="G39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H39">
+        <v>1</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>29</v>
       </c>
@@ -1476,8 +1698,14 @@
       <c r="G41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H41">
+        <v>1</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>22</v>
       </c>
@@ -1499,8 +1727,14 @@
       <c r="G42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H42">
+        <v>1</v>
+      </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>21</v>
       </c>
@@ -1522,8 +1756,14 @@
       <c r="G43">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H43">
+        <v>1</v>
+      </c>
+      <c r="I43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>28</v>
       </c>
@@ -1545,8 +1785,14 @@
       <c r="G44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H44">
+        <v>1</v>
+      </c>
+      <c r="I44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>30</v>
       </c>
@@ -1568,13 +1814,19 @@
       <c r="G45">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H45">
+        <v>1</v>
+      </c>
+      <c r="I45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>34</v>
       </c>
@@ -1596,8 +1848,14 @@
       <c r="G47">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H47">
+        <v>0</v>
+      </c>
+      <c r="I47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>47</v>
       </c>
@@ -1619,8 +1877,14 @@
       <c r="G48">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H48">
+        <v>0</v>
+      </c>
+      <c r="I48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>38</v>
       </c>
@@ -1642,8 +1906,14 @@
       <c r="G49">
         <v>1</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H49">
+        <v>0</v>
+      </c>
+      <c r="I49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>43</v>
       </c>
@@ -1665,8 +1935,14 @@
       <c r="G50">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H50">
+        <v>0</v>
+      </c>
+      <c r="I50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>35</v>
       </c>
@@ -1688,8 +1964,14 @@
       <c r="G51">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H51">
+        <v>0</v>
+      </c>
+      <c r="I51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>61</v>
       </c>
@@ -1711,8 +1993,14 @@
       <c r="G52">
         <v>1</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>33</v>
       </c>
@@ -1734,8 +2022,14 @@
       <c r="G53">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H53">
+        <v>0</v>
+      </c>
+      <c r="I53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>42</v>
       </c>
@@ -1757,8 +2051,14 @@
       <c r="G54">
         <v>1</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H54">
+        <v>0</v>
+      </c>
+      <c r="I54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>37</v>
       </c>
@@ -1780,8 +2080,14 @@
       <c r="G55">
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>46</v>
       </c>
@@ -1803,8 +2109,14 @@
       <c r="G56">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>36</v>
       </c>
@@ -1826,8 +2138,14 @@
       <c r="G57">
         <v>1</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H57">
+        <v>0</v>
+      </c>
+      <c r="I57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>55</v>
       </c>
@@ -1848,6 +2166,12 @@
       </c>
       <c r="G58">
         <v>0</v>
+      </c>
+      <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add NEW! tags, Photo Pop, Welcome Screens typo fix
</commit_message>
<xml_diff>
--- a/source/spreadsheets/BES_NV_Environments_and_Features_for_Claude.xlsx
+++ b/source/spreadsheets/BES_NV_Environments_and_Features_for_Claude.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmestes87/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4213A8AF-0D29-8749-AD2A-1F37610292E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA6D7956-4C10-FD46-A00F-0DFC4288BC3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" xr2:uid="{DB342F5B-931C-1D4F-B9D1-BF0B938CA362}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="65">
   <si>
     <t>Requires Subscription</t>
   </si>
@@ -206,9 +206,6 @@
     <t>BES NV Value</t>
   </si>
   <si>
-    <t>Weleome Screens</t>
-  </si>
-  <si>
     <t>Neo-Fi</t>
   </si>
   <si>
@@ -231,6 +228,12 @@
   </si>
   <si>
     <t>Feature</t>
+  </si>
+  <si>
+    <t>New</t>
+  </si>
+  <si>
+    <t>Welcome Screens</t>
   </si>
 </sst>
 </file>
@@ -611,13 +614,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D87255-3CFF-534A-B67C-04E80AB8E4B8}">
-  <dimension ref="A2:I58"/>
+  <dimension ref="A2:J58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -634,19 +637,22 @@
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I2" t="s">
         <v>62</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -674,8 +680,11 @@
       <c r="I3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>41</v>
       </c>
@@ -703,8 +712,11 @@
       <c r="I4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -732,8 +744,11 @@
       <c r="I5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -761,8 +776,11 @@
       <c r="I6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -790,8 +808,11 @@
       <c r="I7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -819,8 +840,11 @@
       <c r="I8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -848,8 +872,11 @@
       <c r="I9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -877,8 +904,11 @@
       <c r="I10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>44</v>
       </c>
@@ -906,8 +936,11 @@
       <c r="I11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -935,8 +968,11 @@
       <c r="I12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -964,8 +1000,11 @@
       <c r="I13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -993,8 +1032,11 @@
       <c r="I14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -1022,8 +1064,11 @@
       <c r="I15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -1051,8 +1096,11 @@
       <c r="I16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -1080,8 +1128,11 @@
       <c r="I17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -1109,8 +1160,11 @@
       <c r="I18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>40</v>
       </c>
@@ -1138,8 +1192,11 @@
       <c r="I19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -1167,8 +1224,11 @@
       <c r="I20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -1196,8 +1256,11 @@
       <c r="I21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>39</v>
       </c>
@@ -1225,8 +1288,11 @@
       <c r="I22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>7</v>
       </c>
@@ -1254,8 +1320,11 @@
       <c r="I23">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>20</v>
       </c>
@@ -1283,8 +1352,11 @@
       <c r="I24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -1312,8 +1384,11 @@
       <c r="I25">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -1341,8 +1416,11 @@
       <c r="I26">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>11</v>
       </c>
@@ -1370,13 +1448,16 @@
       <c r="I27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>1</v>
       </c>
@@ -1404,8 +1485,11 @@
       <c r="I29">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>50</v>
       </c>
@@ -1433,8 +1517,11 @@
       <c r="I30">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>52</v>
       </c>
@@ -1462,8 +1549,11 @@
       <c r="I31">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>51</v>
       </c>
@@ -1491,8 +1581,11 @@
       <c r="I32">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>49</v>
       </c>
@@ -1520,13 +1613,16 @@
       <c r="I33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>25</v>
       </c>
@@ -1554,8 +1650,11 @@
       <c r="I35">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>31</v>
       </c>
@@ -1583,8 +1682,11 @@
       <c r="I36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>32</v>
       </c>
@@ -1612,8 +1714,11 @@
       <c r="I37">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>27</v>
       </c>
@@ -1641,8 +1746,11 @@
       <c r="I38">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>26</v>
       </c>
@@ -1670,13 +1778,16 @@
       <c r="I39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>29</v>
       </c>
@@ -1704,8 +1815,11 @@
       <c r="I41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>22</v>
       </c>
@@ -1733,8 +1847,11 @@
       <c r="I42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>21</v>
       </c>
@@ -1762,8 +1879,11 @@
       <c r="I43">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>28</v>
       </c>
@@ -1791,8 +1911,11 @@
       <c r="I44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>30</v>
       </c>
@@ -1820,13 +1943,16 @@
       <c r="I45">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>34</v>
       </c>
@@ -1854,8 +1980,11 @@
       <c r="I47">
         <v>1</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>47</v>
       </c>
@@ -1883,8 +2012,11 @@
       <c r="I48">
         <v>1</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>38</v>
       </c>
@@ -1912,8 +2044,11 @@
       <c r="I49">
         <v>1</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>43</v>
       </c>
@@ -1941,8 +2076,11 @@
       <c r="I50">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>35</v>
       </c>
@@ -1970,10 +2108,13 @@
       <c r="I51">
         <v>1</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B52">
         <v>1</v>
@@ -1999,8 +2140,11 @@
       <c r="I52">
         <v>1</v>
       </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>33</v>
       </c>
@@ -2028,8 +2172,11 @@
       <c r="I53">
         <v>1</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>42</v>
       </c>
@@ -2057,8 +2204,11 @@
       <c r="I54">
         <v>1</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>37</v>
       </c>
@@ -2086,8 +2236,11 @@
       <c r="I55">
         <v>1</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>46</v>
       </c>
@@ -2115,8 +2268,11 @@
       <c r="I56">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>36</v>
       </c>
@@ -2144,10 +2300,13 @@
       <c r="I57">
         <v>1</v>
       </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="B58">
         <v>1</v>
@@ -2172,6 +2331,9 @@
       </c>
       <c r="I58">
         <v>1</v>
+      </c>
+      <c r="J58">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Added-since-launch flag toggle for BES NV
</commit_message>
<xml_diff>
--- a/source/spreadsheets/BES_NV_Environments_and_Features_for_Claude.xlsx
+++ b/source/spreadsheets/BES_NV_Environments_and_Features_for_Claude.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cmestes87/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA6D7956-4C10-FD46-A00F-0DFC4288BC3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F16A5FDB-12C8-BC47-A775-ACC5BC6B5224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" xr2:uid="{DB342F5B-931C-1D4F-B9D1-BF0B938CA362}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17820" xr2:uid="{DB342F5B-931C-1D4F-B9D1-BF0B938CA362}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="66">
   <si>
     <t>Requires Subscription</t>
   </si>
@@ -234,6 +234,9 @@
   </si>
   <si>
     <t>Welcome Screens</t>
+  </si>
+  <si>
+    <t>Added After Launch</t>
   </si>
 </sst>
 </file>
@@ -614,13 +617,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D87255-3CFF-534A-B67C-04E80AB8E4B8}">
-  <dimension ref="A2:J58"/>
+  <dimension ref="A2:K58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -637,22 +640,25 @@
         <v>0</v>
       </c>
       <c r="F2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" t="s">
         <v>55</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>59</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>61</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>62</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -669,22 +675,25 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>41</v>
       </c>
@@ -704,19 +713,22 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -736,19 +748,22 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -771,16 +786,19 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -797,7 +815,7 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7">
         <v>1</v>
@@ -806,13 +824,16 @@
         <v>1</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -835,16 +856,19 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -867,16 +891,19 @@
         <v>0</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -899,16 +926,19 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>44</v>
       </c>
@@ -925,22 +955,25 @@
         <v>1</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -963,16 +996,19 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -995,16 +1031,19 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -1021,22 +1060,25 @@
         <v>1</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14">
         <v>0</v>
       </c>
       <c r="H14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -1053,22 +1095,25 @@
         <v>0</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -1085,22 +1130,25 @@
         <v>0</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -1123,16 +1171,19 @@
         <v>0</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -1149,22 +1200,25 @@
         <v>1</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>40</v>
       </c>
@@ -1184,19 +1238,22 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19">
         <v>1</v>
       </c>
       <c r="I19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -1213,22 +1270,25 @@
         <v>0</v>
       </c>
       <c r="F20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -1245,22 +1305,25 @@
         <v>0</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>39</v>
       </c>
@@ -1277,22 +1340,25 @@
         <v>0</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22">
         <v>0</v>
       </c>
       <c r="H22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>7</v>
       </c>
@@ -1309,22 +1375,25 @@
         <v>0</v>
       </c>
       <c r="F23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>20</v>
       </c>
@@ -1347,16 +1416,19 @@
         <v>0</v>
       </c>
       <c r="H24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -1379,16 +1451,19 @@
         <v>0</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -1405,22 +1480,25 @@
         <v>1</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H26">
         <v>1</v>
       </c>
       <c r="I26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>11</v>
       </c>
@@ -1437,7 +1515,7 @@
         <v>0</v>
       </c>
       <c r="F27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G27">
         <v>1</v>
@@ -1446,18 +1524,21 @@
         <v>1</v>
       </c>
       <c r="I27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>1</v>
       </c>
@@ -1474,7 +1555,7 @@
         <v>0</v>
       </c>
       <c r="F29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29">
         <v>1</v>
@@ -1483,13 +1564,16 @@
         <v>1</v>
       </c>
       <c r="I29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J29">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>50</v>
       </c>
@@ -1506,7 +1590,7 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30">
         <v>1</v>
@@ -1515,13 +1599,16 @@
         <v>1</v>
       </c>
       <c r="I30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>52</v>
       </c>
@@ -1541,19 +1628,22 @@
         <v>0</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H31">
         <v>1</v>
       </c>
       <c r="I31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>51</v>
       </c>
@@ -1573,19 +1663,22 @@
         <v>0</v>
       </c>
       <c r="G32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H32">
         <v>1</v>
       </c>
       <c r="I32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>49</v>
       </c>
@@ -1602,27 +1695,30 @@
         <v>1</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H33">
         <v>1</v>
       </c>
       <c r="I33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>25</v>
       </c>
@@ -1645,16 +1741,19 @@
         <v>0</v>
       </c>
       <c r="H35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>31</v>
       </c>
@@ -1677,16 +1776,19 @@
         <v>0</v>
       </c>
       <c r="H36">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>32</v>
       </c>
@@ -1709,16 +1811,19 @@
         <v>0</v>
       </c>
       <c r="H37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>27</v>
       </c>
@@ -1741,16 +1846,19 @@
         <v>0</v>
       </c>
       <c r="H38">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J38">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>26</v>
       </c>
@@ -1773,21 +1881,24 @@
         <v>0</v>
       </c>
       <c r="H39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>29</v>
       </c>
@@ -1810,16 +1921,19 @@
         <v>0</v>
       </c>
       <c r="H41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>22</v>
       </c>
@@ -1842,16 +1956,19 @@
         <v>0</v>
       </c>
       <c r="H42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I42">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>21</v>
       </c>
@@ -1874,16 +1991,19 @@
         <v>0</v>
       </c>
       <c r="H43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J43">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>28</v>
       </c>
@@ -1906,16 +2026,19 @@
         <v>0</v>
       </c>
       <c r="H44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>30</v>
       </c>
@@ -1938,21 +2061,24 @@
         <v>0</v>
       </c>
       <c r="H45">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>34</v>
       </c>
@@ -1978,13 +2104,16 @@
         <v>0</v>
       </c>
       <c r="I47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J47">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="K47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>47</v>
       </c>
@@ -2001,7 +2130,7 @@
         <v>1</v>
       </c>
       <c r="F48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G48">
         <v>0</v>
@@ -2010,13 +2139,16 @@
         <v>0</v>
       </c>
       <c r="I48">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J48">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="K48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>38</v>
       </c>
@@ -2036,19 +2168,22 @@
         <v>0</v>
       </c>
       <c r="G49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J49">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="K49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>43</v>
       </c>
@@ -2065,22 +2200,25 @@
         <v>1</v>
       </c>
       <c r="F50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G50">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I50">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J50">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="K50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>35</v>
       </c>
@@ -2106,13 +2244,16 @@
         <v>0</v>
       </c>
       <c r="I51">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J51">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="K51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>60</v>
       </c>
@@ -2132,19 +2273,22 @@
         <v>0</v>
       </c>
       <c r="G52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H52">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J52">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="K52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>33</v>
       </c>
@@ -2170,13 +2314,16 @@
         <v>0</v>
       </c>
       <c r="I53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J53">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="K53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>42</v>
       </c>
@@ -2196,19 +2343,22 @@
         <v>0</v>
       </c>
       <c r="G54">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H54">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I54">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="K54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>37</v>
       </c>
@@ -2234,13 +2384,16 @@
         <v>0</v>
       </c>
       <c r="I55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="K55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>46</v>
       </c>
@@ -2257,22 +2410,25 @@
         <v>1</v>
       </c>
       <c r="F56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G56">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I56">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J56">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>36</v>
       </c>
@@ -2292,19 +2448,22 @@
         <v>0</v>
       </c>
       <c r="G57">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H57">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I57">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J57">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="K57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>64</v>
       </c>
@@ -2330,14 +2489,17 @@
         <v>0</v>
       </c>
       <c r="I58">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J58">
+        <v>1</v>
+      </c>
+      <c r="K58">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F27">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:G27">
     <sortCondition ref="A3:A27"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>